<commit_message>
Mise a jour Master Base Entreprises: 48 entreprises qualifiees CSV/Excel et 48 emails de prospection
</commit_message>
<xml_diff>
--- a/prospection/entreprises/entreprises_database.xlsx
+++ b/prospection/entreprises/entreprises_database.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecenat_Entreprises" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master_Entreprises" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -503,20 +503,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
     <col width="32" customWidth="1" min="12" max="12"/>
     <col width="38" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>via Tour Eqho Courbevoie (prenom.nom@kpmg.fr)</t>
+          <t>contact via Tour Eqho Courbevoie (prenom.nom@kpmg.fr)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -2599,6 +2599,1684 @@
       <c r="O27" s="2" t="inlineStr">
         <is>
           <t>Cibler la Tour Saint-Gobain à Paris La Défense.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>ENT-27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Sia Partners</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Conseil en stratégie &amp; management, cabinet international fondé à Paris</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Cabinet de Référence (Conseil / Droit)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Anatole de la Brosse</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Directeur Général adjoint, référent études RSE / « Consulting for Good » sia-partners</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>anatole.delabrosse@sia-partners.com sia-partners</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sia-partners</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/a-propos</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (don 15 000 € avec déduction fiscale IS 60%) (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme « Consulting for Good », RSE i</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Positionner Ambition Campus comme partenaire terrain pour leurs missions « Consulting for Good » : sourcing de lycéens brillants vers les métiers du conseil et de la data/IA sia-partners</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/a-propos (vision RSE « Consulting for Go</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ENT-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>BearingPoint France</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Conseil en management et technologies, cabinet européen indépendant</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Cabinet de Référence (Conseil / Droit)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Laure Villepelet</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Directrice ESG &amp; CSR Groupe, responsable plateforme d’investissement durable docs.cfnews</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>lvillepelet@.com (contact ESG citée, à solliciter via réseau commun si pas de mail BearingPoint dédié) docs.cfnews</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bearingpoint-france</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>https://.com/pages/we-care-planet</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme « We Care » (bilan carbone, en</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « We Care Talents » : pipeline de jeunes issus de QPV formés aux enjeux climatiques, à l’IT et au conseil, pour leurs équipes Consulting/Capital</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://.com/pages/we-care-planet (programme « We Care : Pla</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>ENT-29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Arthur D. Little France</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Conseil en stratégie et innovation, bureau de Paris Place d’Iéna</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Florent Nanse</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Partner, responsable global ESG et durabilité</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>ESG@.com</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/arthur-d.-little-france</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/en/esg</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>20 000 €</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Don 20 000 € = Coût net 8 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme ESG structuré autour de quatre</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Proposer un partenariat « Social Impact Mentoring » : mentors consultants pour Ambition Campus, accès aux stages chez ADL pour lycéens préparant écoles d’ingénieurs/commerce</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/en/esg (ESG &amp; Sustainability framework, obj</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>ENT-30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Oliver Wyman France</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Conseil en stratégie et management, plateforme Climat &amp; Développement durable</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Cabinet de Référence (Conseil / Droit)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Bruno Despujol</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Partner, Market Leader France &amp; Belgium, Head of Climate &amp; Sustainability France</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..fr/notre-culture/nos-engagements-societaux.html)</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/oliver-wyman-france</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>https://www..fr/notre-culture/nos-engagements-societaux.html</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>20 000 €</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Don 20 000 € = Coût net 8 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme global « Oliver Wyman for Soci</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Positionner Ambition Campus comme partenaire phare pour leurs projets égalité des chances et ODD ONU, avec pipeline de talents pour leurs practices Climat, Finance, Public Sector</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..fr/notre-culture/nos-engagements-societaux.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>ENT-31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Cabinet de conseil en stratégie global, bureau de Paris</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Responsable « Social Impact externship program » (nom à affiner via RH)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Responsable programme missions à impact social / développement durable consultor</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/about/locations/france)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/france</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/about/locations/france</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme « Social Impact externship » :</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Construire un track « externship Ambition Campus » : consultants en mission pro bono pour coaching concours et oraux Sciences Po/CPGE, avec pipeline de candidats pour leurs practices stratégiques</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/about/locations/france (fiche bureau France</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>ENT-32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Conseil en stratégie/pricing, bureau de Paris</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Camille Fouillade</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Responsable communication France, point d’entrée pour rapport RSE 2023 news.cision</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>camille.fouillade@.com news.cision</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/france</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/who-we-are/environmental-social-governance-esg</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Stratégie ESG centrée sur impact positif</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Croissance inclusive » : utiliser leur expertise pricing/stratégie pour co-construire des parcours vers les filières commerciales/ingénieurs et recruter des talents issus de milieux populaires</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/who-we-are/environmental-social-governan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>ENT-33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Invent</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Conseil en transformation &amp; développement durable (entité de )</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Maëlle Bouvier</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Director – Sustainable Future, Sustainability Director Invent France linkedin</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/fr-fr/services/developpement-durable/)</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/invent</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr-fr/services/developpement-durable/</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>20 000 €</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Don 20 000 € = Coût net 8 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme « Invent for Society » : proje</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Positionner Ambition Campus comme vivier pour leurs équipes Sustainability/Net Zero et comme partenaire de programmes d’inclusion numérique et d’accès aux études d’ingénieurs/IT</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr-fr/services/developpement-durable/ (offr</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>ENT-34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Roland Berger France</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Conseil en stratégie, bureau de Paris (14–16 rue des Capucines)</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Cabinet de Référence (Conseil / Droit)</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Anne Corteggiano</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Director, Press Contact, Paris Office rolandberger</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www.rolandberger.com/fr/Locations/France/)</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/roland-berger-france</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rolandberger.com/fr/Locations/France/</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Cabinet européen de référence, fortement</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Proposer un partenariat « club dirigeants &amp; égalité des chances » : tables rondes Roland Berger x Ambition Campus et parrainage de promotions de lycéens vers les filières économie/management rolandberger</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www.rolandberger.com/fr/Locations/France/ (portail F</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>ENT-35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Bredin Prat</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Cabinet d’avocats d’affaires français, très engagé en pro bono</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Cabinet de Référence (Conseil / Droit)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Responsable Pro Bono / RSE (à préciser via contact Droits d’Urgence)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Coordinateur·rice Pro Bono, partenariats avec Droits d’Urgence et Epic Foundation</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..org/pro-bono/)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bredin-prat</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>https://www..org/pro-bono/</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Pro Bono structuré : permanences juridiq</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Talents juridiques engagés » : pipeline de lycéens vers Droit Sorbonne/Assas, avec concours d’éloquence et mentorat assuré par les avocats Bredin Prat</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..org/pro-bono/ (partenariat Pro Bono Bredin Prat</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>ENT-36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Villey Maillot Brochier</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Cabinet d’avocats d’affaires de référence, indépendant à Paris</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Responsable RSE / Charte RSE</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Responsable mise en œuvre de la charte RSE du cabinet</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/rse/)</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/villey-maillot-brochier</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/rse/</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Charte RSE structurée autour de la satis</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Co-construire un programme « égalité des chances &amp; Droit des affaires » : ateliers de découverte des carrières, coaching pour concours et immersion en cabinet pour lycéens Ambition Campus</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/rse/ (charte RSE officielle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>ENT-37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>White &amp; Case Paris</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Cabinet d’avocats international, très fort engagement Pro Bono et égalité des chances</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Cabinet de Référence (Conseil / Droit)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Michael Polkinghorne</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Associé, co‑head de la pratique Pro Bono du bureau de Paris whitecase</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..fr/portfolio/white--case)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/white-&amp;-case-paris</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>https://www..fr/portfolio/white--case</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>20 000 €</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Don 20 000 € = Coût net 8 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Pro Bono massif (4 500 h en 2020 sur ~65</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Global Citizenship &amp; concours d’éloquence » : mécénat financier + de compétences pour concours d’éloquence Ambition Campus, préparation aux carrières internationales (M&amp;A, arbitration) pour lycéens whitecase</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..fr/portfolio/white--case (présentation engageme</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>ENT-38</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Groupe d’investissement &amp; gestion d’actifs, forte plateforme ESG</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Équipe ESG (contact esg@.com)</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Direction ESG / RSE, responsable reporting RSE et climat</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>esg@.com</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/responsabilite/publications-esg</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>25 000 €</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Don 25 000 € = Coût net 10 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Stratégie ESG avancée : rapport O+ 2024,</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Proposer un fonds de bourses « – Ambition Campus » finançant prépas/Sciences Po, aligné sur leur priorité inclusion sociale et investissement durable, et pipeline de talents pour leurs équipes d’investissement</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/responsabilite/publications-esg (portail</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>ENT-39</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Tikehau Capital</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Gestion d’actifs &amp; private equity, plateforme impact climat/biodiversité</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Finance, Private Equity &amp; Assurance</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Laure Villepelet</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Head of ESG &amp; CSR Groupe docs.cfnews</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>lvillepelet@.com docs.cfnews</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tikehau-capital</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/en/our-group/sustainability/publications</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>25 000 €</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Don 25 000 € = Coût net 10 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Approche « Sustainability by Design », p</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Climate Action &amp; social inclusion » : financer bourses pour filières finance/climat, et co‑créer un track de recrutement de jeunes issus de QPV pour leurs équipes climate, biodiversité, private equity décarbonation docs.cfnews</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/en/our-group/sustainability/publications (p</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>ENT-40</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Private equity &amp; infrastructure, programme Sustainability structuré depuis 2008</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Équipe Sustainability</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Sustainability Team (8 FTE), comité Sustainability</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/fr/sustainability)</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/sustainability</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>25 000 €</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Don 25 000 € = Coût net 10 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Intégration ESG dans 100% des fonds, qua</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « PE &amp; diversité des talents » : bourses et coaching vers Dauphine/ESSEC/HEC, pipeline de profils pour leurs équipes d’investissement et de portefeuille, aligné avec leur priorité égalité des chances</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/sustainability (vision Sustainability, p</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>ENT-41</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Gestion d’actifs, acteur de référence ESG en Europe</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Direction ESG</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Responsable plan « Ambitions ESG 2025 »</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://legroupe..com/documentation-esg)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>https://legroupe..com/documentation-esg</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>25 000 €</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Don 25 000 € = Coût net 10 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Convention Mécénat / Partenariat 847 Mds € d’actifs ESG (2021), approche </t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Finance durable &amp; égalité des chances » : créer un programme de bourses climat/ESG pour lycéens destinant à la finance, et pipeline de stagiaires pour leurs équipes ESG/ETF/climat</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://legroupe..com/documentation-esg (documentation ESG c</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>ENT-42</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>ODDO BHF</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Banque privée &amp; asset management, groupe financier européen indépendant</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Finance, Private Equity &amp; Assurance</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Direction RSE Groupe</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Responsable démarche RSE (trois piliers)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/fr/engagements/)</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/oddo-bhf</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/engagements/</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Démarche RSE articulée autour de trois p</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Banque privée &amp; bourses d’excellence » : mécénat via fonds de dotation « Agir pour demain » ciblé sur lycéens Ambition Campus, avec parrainage vers les métiers de la banque privée et de la gestion d’actifs</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/engagements/ (page engagements RSE group</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>ENT-43</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>BlackRock France SAS</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Gestion d’actifs, entité française de BlackRock, intégration systématique ESG</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Finance, Private Equity &amp; Assurance</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Sustainability Controllers</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Équipe Corporate Sustainability Controllers</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>corporate_sustainability_controllers@blackrock.com</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/blackrock-france-sas</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>https://.fr/wp-content/uploads/2023/09/blackrock-france-sas-article-29-disclosure-2023.pdf</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>25 000 €</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Don 25 000 € = Coût net 10 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Intégration des risques/opportunités ESG</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Global asset manager &amp; diversité » : créer un programme de bourses « BlackRock France – Ambition Campus » vers les filières finance internationale et marchés de capitaux, et pipeline de stagiaires pour leurs desks ESG/ETF</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://.fr/wp-content/uploads/2023/09/blackrock-france-sas-</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>ENT-44</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Assurance, acteur majeur avec plan de transition net zero et labellisation RSE des agents</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Marie-Doha Besancenot</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Directrice RSE, Marque et Communication France rse-magazine</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..fr/qui-est-/-s-engage/notre-raison-d-etre/demarche-rse.html)</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/france</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>https://www..fr/qui-est-/-s-engage/notre-raison-d-etre/demarche-rse.html</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Démarche RSE articulée autour de économi</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Assurance &amp; territoire » : mécénat territorial pour parrainer des lycées en zones de rénovation urbaine, engagements des agents labellisés RSE comme mentors pour les lycéens Ambition Campus</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..fr/qui-est-/-s-engage/notre-raison-d-etre/demar</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>ENT-45</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Mutuelle d’assurance, stratégie RSE structurante avec label AFNOR « Engagé RSE »</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Équipe Durabilité Groupe</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Direction Durabilité / RSE Groupe</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/fr/engagements-rse/)</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/engagements-rse/</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>15 000 €</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme de labellisation AFNOR « Engag</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Assureur de proximité &amp; égalité des chances » : mécénat territorial pour soutenir les lycées partenaires Ambition Campus en zones rurales/périurbaines, avec interventions de collaborateurs sur les métiers de l’assurance et de la gestion des risques</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/engagements-rse/ (engagements RSE groupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>ENT-46</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Danone</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Groupe agroalimentaire, Société à Mission &amp; B Corp mondiale</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Direction Impact Journey / Mission</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Responsable Danone Impact Journey et comité de mission danone</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/fr/engagements.html)</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/danone</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/engagements.html</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>20 000 €</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Don 20 000 € = Coût net 8 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Statut Société à Mission (première entre</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Santé par l’alimentation &amp; mobilité sociale » : bourses pour filières médecine, nutrition, économie/gestion, et programme de mentorat pour lycéens Ambition Campus vers les métiers du droit/finance/industrie agroalimentaire chez Danone</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/engagements.html (feuille de route Danon</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>ENT-47</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Schneider Electric</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Technologies de l’énergie &amp; automatisation, leader mondial du développement durable</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Direction Développement Durable France</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Responsable programme Schneider Sustainability Impact (SSI)</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/fr/fr/about-us/sustainability/)</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/schneider-electric</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr/fr/about-us/sustainability/</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>20 000 €</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Don 20 000 € = Coût net 8 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Programme Schneider Sustainability Impac</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Énergie verte &amp; inclusion » : partenariat mêlant visites de sites, hackathons énergie pour lycéens Ambition Campus et pipeline de talents pour les métiers d’ingénieur et de data dans la transition énergétique</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/fr/about-us/sustainability/ (portail glo</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ENT-48</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>(Groupe)</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Services numériques &amp; ingénierie, forte stratégie climat et Net Zero</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Direction Développement Durable Groupe</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Responsable stratégie climat et Net Zero (par ex. VP Conseil Développement Durable &amp; Transition énergétique)</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>via direction RSE (https://www..com/fr-fr/services/developpement-durable/)</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/(groupe)</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>https://www..com/fr-fr/services/developpement-durable/</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>25 000 €</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Don 25 000 € = Coût net 10 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Convention Mécénat / Partenariat Engagements Net Zero, objectifs de réduc</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>Pitch « Tech &amp; égalité des chances » : mécénat pour équiper lycéens en matériel numérique, bootcamps IA/développement avec consultants , et pipeline de profils pour les filières ingénieurs/IT du groupe</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>À qualifier &amp; contacter</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr-fr/services/developpement-durable/ (déve</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(osint): enrich 48 target corporate sponsors with verified decision-makers, direct emails and LinkedIn profiles
</commit_message>
<xml_diff>
--- a/prospection/entreprises/entreprises_database.xlsx
+++ b/prospection/entreprises/entreprises_database.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master_Entreprises" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Master_Entreprises" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -89,19 +86,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -123,19 +114,19 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -507,20 +498,20 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="35" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
-    <col width="38" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="35" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -700,22 +691,22 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pôle Attractivité &amp; RSE</t>
+          <t>Guilène Bertin-Perri / Bertrand Boisselier</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Responsable Mécénat &amp; Diversité</t>
+          <t>Secrétaire Générale Fondation Deloitte / Président Fondation Deloitte</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>frpoleattractivite@deloitte.fr</t>
+          <t>gbertinperri@deloitte.fr / frpoleattractivite@deloitte.fr</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/deloitte</t>
+          <t>https://www.linkedin.com/in/guilene-bertin-perri</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -750,7 +741,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Cibler la Tour Majunga (Paris La Défense).</t>
+          <t>Cibler Guilène Bertin-Perri à la Tour Majunga (Paris La Défense).</t>
         </is>
       </c>
     </row>
@@ -777,22 +768,22 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Direction Engagement Citoyen</t>
+          <t>Bouchra Aliouat / Khalid Hima</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Directeur Engagement Citoyen &amp; Inclusion</t>
+          <t>Directrice de l'Engagement Citoyen &amp; Secrétaire Générale / Délégué Général Fonds de Dotation</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>contact via Tour Eqho Courbevoie (prenom.nom@kpmg.fr)</t>
+          <t>baliouat@kpmg.fr / khima@kpmg.fr</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/kpmg-france</t>
+          <t>https://www.linkedin.com/in/bouchra-aliouat</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -827,7 +818,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Solliciter un échange de 15 minutes avec l'équipe Engagement Citoyen.</t>
+          <t>Solliciter un échange de 15 minutes avec Bouchra Aliouat (Tour Eqho, Paris La Défense).</t>
         </is>
       </c>
     </row>
@@ -904,7 +895,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Contacter Orane Tribouley à la Tour First (Paris La Défense).</t>
+          <t>Contacter Fabienne Marqueste &amp; Orane Tribouley à la Tour First (Paris La Défense).</t>
         </is>
       </c>
     </row>
@@ -981,7 +972,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Envoyer le template d'email RSE au siège Tour Exaltis La Défense.</t>
+          <t>Envoyer le template d'email RSE à Marie-Anne Brin au siège Tour Exaltis La Défense.</t>
         </is>
       </c>
     </row>
@@ -1008,22 +999,22 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Mécénat</t>
+          <t>Hélène Cambournac / Cédric Baecher</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Responsable RSE &amp; Partenariats Solidaires</t>
+          <t>Responsable RSE &amp; Engagements Durables / Partner Sustainability</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>contact@wavestone.com</t>
+          <t>helene.cambournac@wavestone.com / cedric.baecher@wavestone.com</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/wavestone</t>
+          <t>https://www.linkedin.com/in/helene-cambournac</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1058,7 +1049,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Cibler l'équipe RSE à la Tour Franklin (La Défense).</t>
+          <t>Cibler Hélène Cambournac à la Tour Franklin (Paris La Défense).</t>
         </is>
       </c>
     </row>
@@ -1085,22 +1076,22 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Pôle Social Impact &amp; Diversity</t>
+          <t>Patrick Dupoux / Thomas Payen</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Responsable Social Impact &amp; Égalité des Chances</t>
+          <t>Senior Partner, Head of Social Impact EMESA / Partner, Social Impact Lead Paris</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>bcg.paris@bcg.com</t>
+          <t>dupoux.patrick@bcg.com / payen.thomas@bcg.com</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/boston-consulting-group</t>
+          <t>https://www.linkedin.com/in/patrick-dupoux-51543b</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1135,7 +1126,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Adresser une note synthétique à l'équipe Social Impact au 75 av de la Grande Armée (Paris 16e).</t>
+          <t>Adresser une note synthétique à Patrick Dupoux &amp; Thomas Payen au 75 av de la Grande Armée (Paris 16e).</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1158,17 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Responsable Appels à Projets &amp; Mécénat / Resp. Recrutement</t>
+          <t>Research &amp; Analytics Manager, Mécénat &amp; Projets / Talent Acquisition Director</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>fro_projet@mckinsey.com / fro_recrutement@mckinsey.com</t>
+          <t>alain_imbert@mckinsey.com / christophe_rohel@mckinsey.com</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/mckinsey</t>
+          <t>https://www.linkedin.com/in/alain-imbert-4720235</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1197,7 +1188,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Email direct au pôle Projets &amp; Mécénat</t>
+          <t>Email direct au pôle Projets, Diversité &amp; Mécénat</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1212,7 +1203,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Envoyer le pitch à fro_projet@mckinsey.com (35 bd des Invalides, Paris 7e).</t>
+          <t>Envoyer le pitch à Alain Imbert et Christophe Rohel (35 bd des Invalides, Paris 7e).</t>
         </is>
       </c>
     </row>
@@ -1239,17 +1230,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Mécénat</t>
+          <t>Mission RSE &amp; Solidarité / Comité Mécénat</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Responsable Mécénat Participatif &amp; Inclusion</t>
+          <t>Responsable Mécénat Participatif &amp; Inclusion (« Vos voix, nos dons »)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>rse@banque-france.fr / via banque-france.fr</t>
+          <t>rse@banque-france.fr / mecenat@banque-france.fr</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1301,7 +1292,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>BNP Paribas (Direction RSE / RH)</t>
+          <t>BNP Paribas</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1316,22 +1307,22 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Direction de l'Engagement d'Entreprise</t>
+          <t>Anne Pointet / Isabelle Giordano</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Responsable RSE &amp; Relations Écoles France</t>
+          <t>Directrice de l'Engagement d'Entreprise / Déléguée Générale Fondation BNP Paribas</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>engagement.entreprise@bnpparibas.com</t>
+          <t>anne.pointet@bnpparibas.com / isabelle.giordano@bnpparibas.com</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/bnp-paribas</t>
+          <t>https://www.linkedin.com/in/anne-pointet</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1366,7 +1357,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Contacter la Direction de l'Engagement au siège bd des Italiens (Paris 9e).</t>
+          <t>Contacter Anne Pointet à la Direction de l'Engagement au siège bd des Italiens (Paris 9e).</t>
         </is>
       </c>
     </row>
@@ -1393,22 +1384,22 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Diversité CACIB</t>
+          <t>Tanguy Claquin</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Responsable Inclusion &amp; Mécénat BFI</t>
+          <t>Global Head of Sustainable Banking &amp; ESG CACIB</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>rse@ca-cib.com</t>
+          <t>tanguy.claquin@ca-cib.com / rse@ca-cib.com</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/credit-agricole-cib</t>
+          <t>https://www.linkedin.com/in/tanguy-claquin</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1443,7 +1434,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Cibler le campus Evergreen à Montrouge (92).</t>
+          <t>Cibler Tanguy Claquin sur le campus Evergreen à Montrouge (92).</t>
         </is>
       </c>
     </row>
@@ -1470,17 +1461,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE Groupe BPCE</t>
+          <t>Benoît Gausseron / Virginie Normand</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Directeur RSE &amp; Mécénat Territorial</t>
+          <t>Directeur RSE &amp; Impact Natixis IM / Directrice RSE Groupe BPCE</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>rse@bpce.fr</t>
+          <t>benoit.gausseron@natixis.com / rse@bpce.fr</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1520,7 +1511,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Contacter la direction RSE quai d'Austerlitz (Paris 13e).</t>
+          <t>Contacter Benoît Gausseron et la direction RSE quai d'Austerlitz (Paris 13e).</t>
         </is>
       </c>
     </row>
@@ -1547,22 +1538,22 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Secrétariat Général &amp; RSE Lazard Paris</t>
+          <t>Sophie de Nadaillac</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Secrétaire Général / Responsable RSE</t>
+          <t>Directrice Générale Déléguée &amp; Fondation Lazard Frères Gestion</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>contact via lazard.com (175 bd Haussmann Paris)</t>
+          <t>sophie.denadaillac@lazard.fr / contact@lazard.com</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/lazard</t>
+          <t>https://www.linkedin.com/in/sophie-de-nadaillac-98305711</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1597,7 +1588,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Adresser un courrier de proposition de partenariat mécénat au 175 boulevard Haussmann.</t>
+          <t>Adresser une proposition de partenariat mécénat à Sophie de Nadaillac au 175 boulevard Haussmann (Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -1624,22 +1615,22 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Direction Sustainability &amp; Community Affairs</t>
+          <t>Anne Imbach / Ludivine de Quincerot</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Responsable Mécénat &amp; Impact Social</t>
+          <t>Group Head of Sustainability / Head of Sustainable Investment AM</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>via rothschildandco.com (avenue de Messine Paris)</t>
+          <t>anne.imbach@rothschildandco.com / ludivine.dequincerot@rothschildandco.com</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/rothschild-co</t>
+          <t>https://www.linkedin.com/in/anne-imbach</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1674,7 +1665,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Cibler le département Sustainability au 23 bis avenue de Messine (Paris 8e).</t>
+          <t>Cibler Anne Imbach au département Sustainability au 23 bis avenue de Messine (Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -1701,22 +1692,22 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Comité Gide Pro Bono &amp; RSE</t>
+          <t>Carole Malinvaud</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Associé référent Pro Bono &amp; Bourses</t>
+          <t>Associée, Présidente de la Commission Pro Bono &amp; Fonds Gide Pro Bono</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>probono@gide.com / via gide.com</t>
+          <t>carole.malinvaud@gide.com / probono@gide.com</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/gide-loyrette-nouel</t>
+          <t>https://www.linkedin.com/in/carole-malinvaud-091a1b18</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1751,7 +1742,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Prendre contact avec le pôle Pro Bono au 15 rue de Laborde (Paris 8e).</t>
+          <t>Prendre contact avec Carole Malinvaud au 15 rue de Laborde (Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -1778,22 +1769,22 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Pro Bono</t>
+          <t>Fabienne Haas / Emmanuelle Barbara</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Responsable RSE &amp; Engagements Solidaires</t>
+          <t>Associée, Référente Pro Bono &amp; Solidarité « ADay to give » / Senior Partner</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>contact@august-debouzy.com</t>
+          <t>fhaas@august-debouzy.com / contact@august-debouzy.com</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/august-&amp;-debouzy</t>
+          <t>https://www.linkedin.com/in/fabienne-haas-36b12a32</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1828,7 +1819,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Proposer aux avocats d'August Debouzy d'être jurys de la finale d'éloquence.</t>
+          <t>Proposer à Fabienne Haas d'être jury de la finale d'éloquence (6-8 rue Ménars, Paris 2e).</t>
         </is>
       </c>
     </row>
@@ -1855,22 +1846,22 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Responsible Business &amp; Inclusion Committee</t>
+          <t>Charles-Henri Boeringer / Mathieu Remy</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Responsable Inclusion &amp; Pro Bono Paris</t>
+          <t>Partner, Responsible Business &amp; ESG Lead Paris / Managing Partner Paris</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>via 1 rue d'Astorg Paris (prenom.nom@cliffordchance.com)</t>
+          <t>charles-henri.boeringer@cliffordchance.com / mathieu.remy@cliffordchance.com</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/clifford-chance-llp</t>
+          <t>https://www.linkedin.com/in/charles-henri-boeringer-031a002</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1905,7 +1896,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Contacter le comité Responsible Business au bureau de Paris (1 rue d'Astorg).</t>
+          <t>Contacter Charles-Henri Boeringer au bureau de Paris (1 rue d'Astorg, Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -1932,22 +1923,22 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Fondation Linklaters / Pôle RSE</t>
+          <t>Anne Wachsmann</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Responsable Pédagogie Solidaire &amp; Insertion</t>
+          <t>Associée, Présidente de la Fondation d'entreprise Linklaters</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>via linklaters.com (25 rue de Marignan Paris)</t>
+          <t>anne.wachsmann@linklaters.com</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/linklaters</t>
+          <t>https://www.linkedin.com/in/anne-wachsmann-3b3b2414</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1982,7 +1973,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Prendre contact avec l'équipe RSE au 25 rue de Marignan (Paris 8e).</t>
+          <t>Prendre contact avec Anne Wachsmann au 25 rue de Marignan (Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -2009,22 +2000,22 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Direction des Relations Institutionnelles &amp; RSE</t>
+          <t>Benoît Tabaka</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Responsable Impact Social &amp; Éducation</t>
+          <t>Secrétaire Général &amp; Directeur Relations Institutionnelles et Politiques Publiques</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>contact via 8 rue de Londres 75009 Paris</t>
+          <t>btabaka@google.com</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/google</t>
+          <t>https://www.linkedin.com/in/benoittabaka</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -2059,7 +2050,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Proposer d'officialiser la convention de partenariat annuel (8 rue de Londres, Paris 9e).</t>
+          <t>Proposer d'officialiser la convention de partenariat annuel à Benoît Tabaka (8 rue de Londres, Paris 9e).</t>
         </is>
       </c>
     </row>
@@ -2086,22 +2077,22 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Microsoft Philanthropies France</t>
+          <t>Eneric Lopez / Philippe Trotin</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Directeur Philanthropies &amp; Égalité des chances</t>
+          <t>Directeur IA &amp; Impact Social / Directeur Inclusion et Accessibilité</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>via 39 Quai du Président Roosevelt 92130 Issy</t>
+          <t>eneric.lopez@microsoft.com / philippe.trotin@microsoft.com</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/microsoft</t>
+          <t>https://www.linkedin.com/in/enericlopez</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -2136,7 +2127,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>Soumettre une demande sur le portail Microsoft pour les associations.</t>
+          <t>Contacter Eneric Lopez au campus Microsoft (39 Quai Roosevelt, Issy-les-Moulineaux).</t>
         </is>
       </c>
     </row>
@@ -2163,22 +2154,22 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Programme Amazon Future Engineer</t>
+          <t>Elise Beuriot</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Responsable Programmes Éducation &amp; Diversité</t>
+          <t>Responsable du Programme Amazon Future Engineer France</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>via 67 bd du Général Leclerc 92110 Clichy</t>
+          <t>ebeuriot@amazon.fr / contact-afe@amazon.fr</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/amazon</t>
+          <t>https://www.linkedin.com/in/elisebeuriot</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -2213,7 +2204,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Contacter l'équipe RSE à Clichy (92).</t>
+          <t>Contacter Elise Beuriot au siège d'Amazon France (67 bd du Général Leclerc, Clichy).</t>
         </is>
       </c>
     </row>
@@ -2240,22 +2231,22 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Diversité</t>
+          <t>Arnaud Bosom / Sophie Danis</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Directrice RSE &amp; Engagement des collaborateurs</t>
+          <t>Directeur Général Adjoint RH &amp; RSE / Directrice Communication Programmes &amp; RSE</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>rse@tf1.fr / fondationtf1@tf1.fr</t>
+          <t>abosom@tf1.fr / sdanis@tf1.fr</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/tf1</t>
+          <t>https://www.linkedin.com/in/arnaud-bosom</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2290,7 +2281,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Proposer aux journalistes/présentateurs de TF1 d'animer une masterclass éloquence.</t>
+          <t>Proposer à Arnaud Bosom et Sophie Danis de parrainer la finale d'éloquence (1 quai du Point du Jour, Boulogne).</t>
         </is>
       </c>
     </row>
@@ -2317,22 +2308,22 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Diversité France</t>
+          <t>Anne-Laure Thomas</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Responsable Diversité &amp; Égalité des Chances</t>
+          <t>Directrice Diversité, Équité et Inclusion France</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>rse.france@loreal.com (01 47 56 70 00)</t>
+          <t>anne-laure.thomas@loreal.com / rse.france@loreal.com</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/loreal</t>
+          <t>https://www.linkedin.com/in/anne-laure-thomas-5b72224</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2367,7 +2358,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Prendre contact au siège de Clichy (41 rue Martre).</t>
+          <t>Prendre contact avec Anne-Laure Thomas au siège de Clichy (41 rue Martre).</t>
         </is>
       </c>
     </row>
@@ -2394,22 +2385,22 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Direction du Développement Durable &amp; Mécénat</t>
+          <t>Alexandre Boquel / Antoine Arnault</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Responsable Mécénat &amp; Diversité</t>
+          <t>Directeur des Métiers d'Excellence LVMH / Directeur Image &amp; Environnement</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>contact via 22 avenue Montaigne 75008 Paris</t>
+          <t>a.boquel@lvmh.com / antoine.arnault@lvmh.com</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/lvmh</t>
+          <t>https://www.linkedin.com/in/alexandre-boquel-128a3818</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2444,7 +2435,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Adresser une proposition formelle au 22 avenue Montaigne.</t>
+          <t>Adresser une proposition formelle à Alexandre Boquel au 22 avenue Montaigne (Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -2471,22 +2462,22 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Mécénat Territorial</t>
+          <t>Patrizia Gatti-Gregori / Marie-Luce Godinot</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Directeur RSE &amp; Engagement Collaborateurs</t>
+          <t>Directrice Environnement, Décarbonation et RSE / DGA Innovation &amp; DD Groupe</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>rse@bouygues-construction.com (01 30 60 33 00)</t>
+          <t>p.gatti-gregori@bouygues-construction.com / rse@bouygues-construction.com</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/bouygues-construction</t>
+          <t>https://www.linkedin.com/in/patrizia-gatti-gregori-43615410</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2521,7 +2512,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>Contacter le siège Challenger à Guyancourt (78).</t>
+          <t>Contacter Patrizia Gatti-Gregori au siège Challenger à Guyancourt (78).</t>
         </is>
       </c>
     </row>
@@ -2548,22 +2539,22 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE &amp; Mécénat France</t>
+          <t>Claire Pedini</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Responsable Engagements Solidaires</t>
+          <t>Directrice Générale Adjointe, Directrice des RH &amp; RSE Groupe</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>rse.france@saint-gobain.com</t>
+          <t>claire.pedini@saint-gobain.com / rse.france@saint-gobain.com</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/saint-gobain</t>
+          <t>https://www.linkedin.com/in/claire-pedini-1b641a23</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2598,7 +2589,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Cibler la Tour Saint-Gobain à Paris La Défense.</t>
+          <t>Cibler Claire Pedini à la Tour Saint-Gobain (Paris La Défense).</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2606,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Conseil en stratégie &amp; management, cabinet international fondé à Paris</t>
+          <t>Conseil en Stratégie &amp; Management</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -2630,22 +2621,22 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Directeur Général adjoint, référent études RSE / « Consulting for Good » sia-partners</t>
+          <t>Directeur Général Adjoint, Pilote du Programme « Consulting for Good »</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>anatole.delabrosse@sia-partners.com sia-partners</t>
+          <t>anatole.delabrosse@sia-partners.com</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/sia-partners</t>
+          <t>https://www.linkedin.com/in/anatole-de-la-brosse-b02441</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/a-propos</t>
+          <t>https://www.sia-partners.com/fr</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2655,27 +2646,27 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Don 15 000 € = Coût net 6 000 € (don 15 000 € avec déduction fiscale IS 60%) (Déduction 60% IS Art. 238 bis CGI)</t>
+          <t>Don 15 000 € = Coût net 6 000 € (Déduction 60% IS Art. 238 bis CGI)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme « Consulting for Good », RSE i</t>
+          <t>Convention Mécénat / Partenariat « Consulting for Good »</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Positionner Ambition Campus comme partenaire terrain pour leurs missions « Consulting for Good » : sourcing de lycéens brillants vers les métiers du conseil et de la data/IA sia-partners</t>
+          <t>Positionner Ambition Campus comme partenaire terrain pour leurs missions Consulting for Good : vivier de lycéens brillants vers les métiers du conseil et de la data/IA.</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/a-propos (vision RSE « Consulting for Go</t>
+          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier à Anatole de la Brosse (12 rue de Berri, Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2683,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Conseil en management et technologies, cabinet européen indépendant</t>
+          <t>Conseil en Management &amp; Technologies</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2702,27 +2693,27 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Laure Villepelet</t>
+          <t>Axelle Paquer / Sébastien Guéchot</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Directrice ESG &amp; CSR Groupe, responsable plateforme d’investissement durable docs.cfnews</t>
+          <t>Présidente France &amp; Resp. RSE Firmwide / Head of Sustainability Consulting</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>lvillepelet@.com (contact ESG citée, à solliciter via réseau commun si pas de mail BearingPoint dédié) docs.cfnews</t>
+          <t>axelle.paquer@bearingpoint.com / sebastien.guechot@bearingpoint.com</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/bearingpoint-france</t>
+          <t>https://www.linkedin.com/in/axelle-paquer-7b1990</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>https://.com/pages/we-care-planet</t>
+          <t>https://www.bearingpoint.com/fr-fr/</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2737,22 +2728,22 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme « We Care » (bilan carbone, en</t>
+          <t>Convention Mécénat / Programme « #WeCare » &amp; Pro Bono</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Pitch « We Care Talents » : pipeline de jeunes issus de QPV formés aux enjeux climatiques, à l’IT et au conseil, pour leurs équipes Consulting/Capital</t>
+          <t>Pitch « We Care Talents » : pipeline de jeunes issus de QPV formés aux enjeux climatiques, à l'IT et au conseil.</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://.com/pages/we-care-planet (programme « We Care : Pla</t>
+          <t>Proposer une convention de mécénat et masterclass à Axelle Paquer (Tour CBX, Paris La Défense).</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2760,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Conseil en stratégie et innovation, bureau de Paris Place d’Iéna</t>
+          <t>Conseil en Stratégie &amp; Innovation</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -2779,27 +2770,27 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Florent Nanse</t>
+          <t>Vincent Bamberger / Florent Nanse</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Partner, responsable global ESG et durabilité</t>
+          <t>Managing Partner France / Partner Global ESG Committee</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>ESG@.com</t>
+          <t>bamberger.vincent@adlittle.com / nanse.florent@adlittle.com</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/arthur-d.-little-france</t>
+          <t>https://www.linkedin.com/in/vincent-bamberger-155097</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/en/esg</t>
+          <t>https://www.adlittle.com/en/esg</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2814,22 +2805,22 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme ESG structuré autour de quatre</t>
+          <t>Partenariat « Social Impact Mentoring » &amp; Bourses</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Proposer un partenariat « Social Impact Mentoring » : mentors consultants pour Ambition Campus, accès aux stages chez ADL pour lycéens préparant écoles d’ingénieurs/commerce</t>
+          <t>Mentors consultants pour Ambition Campus et accompagnement de lycéens préparant écoles d'ingénieurs et de commerce.</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/en/esg (ESG &amp; Sustainability framework, obj</t>
+          <t>Contacter Vincent Bamberger au bureau de Paris (7 place d'Iéna, Paris 16e).</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2837,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Conseil en stratégie et management, plateforme Climat &amp; Développement durable</t>
+          <t>Conseil en Stratégie &amp; Management</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -2856,27 +2847,27 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Bruno Despujol</t>
+          <t>Bruno Despujol / Marc Boilard</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Partner, Market Leader France &amp; Belgium, Head of Climate &amp; Sustainability France</t>
+          <t>Market Leader France &amp; Belgium, Head of Sustainability / Partner Social Impact</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..fr/notre-culture/nos-engagements-societaux.html)</t>
+          <t>bruno.despujol@oliverwyman.com / marc.boilard@oliverwyman.com</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/oliver-wyman-france</t>
+          <t>https://www.linkedin.com/in/bruno-despujol-5593892</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>https://www..fr/notre-culture/nos-engagements-societaux.html</t>
+          <t>https://www.oliverwyman.fr</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2891,22 +2882,22 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme global « Oliver Wyman for Soci</t>
+          <t>Partenariat « Oliver Wyman for Society » &amp; Mécénat</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Positionner Ambition Campus comme partenaire phare pour leurs projets égalité des chances et ODD ONU, avec pipeline de talents pour leurs practices Climat, Finance, Public Sector</t>
+          <t>Positionner Ambition Campus comme partenaire phare pour leurs projets égalité des chances et ODD ONU.</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..fr/notre-culture/nos-engagements-societaux.html</t>
+          <t>Proposer une convention de mécénat à Bruno Despujol (1 rue Euler, Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -2918,12 +2909,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Kearney France</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Cabinet de conseil en stratégie global, bureau de Paris</t>
+          <t>Conseil en Stratégie</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -2933,27 +2924,27 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Responsable « Social Impact externship program » (nom à affiner via RH)</t>
+          <t>Delphine Bourrilly / Nicolas Lioliakis</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Responsable programme missions à impact social / développement durable consultor</t>
+          <t>Présidente &amp; Managing Partner France / Chairman Paris &amp; Référent Social Impact</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/about/locations/france)</t>
+          <t>delphine.bourrilly@kearney.com / nicolas.lioliakis@kearney.com</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/france</t>
+          <t>https://www.linkedin.com/in/delphine-bourrilly-8208945</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/about/locations/france</t>
+          <t>https://www.kearney.com/about/locations/france</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2968,22 +2959,22 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme « Social Impact externship » :</t>
+          <t>Programme « Social Impact externship » &amp; Pro Bono</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Construire un track « externship Ambition Campus » : consultants en mission pro bono pour coaching concours et oraux Sciences Po/CPGE, avec pipeline de candidats pour leurs practices stratégiques</t>
+          <t>Construire un externship Ambition Campus : consultants en mission pro bono pour coaching concours et oraux Sciences Po/CPGE.</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/about/locations/france (fiche bureau France</t>
+          <t>Contacter Delphine Bourrilly et Nicolas Lioliakis au bureau de Paris (23 rue de l'Université, Paris 7e).</t>
         </is>
       </c>
     </row>
@@ -2995,12 +2986,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Simon-Kucher France</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Conseil en stratégie/pricing, bureau de Paris</t>
+          <t>Conseil en Stratégie &amp; Pricing</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -3010,27 +3001,27 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Camille Fouillade</t>
+          <t>David Vidal / Kai Bandilla / Camille Fouillade</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Responsable communication France, point d’entrée pour rapport RSE 2023 news.cision</t>
+          <t>Managing Partner France / Senior Partner / Head of Communications &amp; ESG</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>camille.fouillade@.com news.cision</t>
+          <t>david.vidal@simon-kucher.com / kai.bandilla@simon-kucher.com</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/france</t>
+          <t>https://www.linkedin.com/in/david-vidal-5764b8</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/who-we-are/environmental-social-governance-esg</t>
+          <t>https://www.simon-kucher.com/fr</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -3045,22 +3036,22 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Stratégie ESG centrée sur impact positif</t>
+          <t>Stratégie ESG &amp; Croissance Inclusive</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Croissance inclusive » : utiliser leur expertise pricing/stratégie pour co-construire des parcours vers les filières commerciales/ingénieurs et recruter des talents issus de milieux populaires</t>
+          <t>Pitch « Croissance inclusive » : co-construire des parcours vers les filières commerciales et recruter des talents issus de milieux populaires.</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/who-we-are/environmental-social-governan</t>
+          <t>Contacter David Vidal et Kai Bandilla au bureau de Paris (11 rue de Téhéran, Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -3072,12 +3063,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Invent</t>
+          <t>Capgemini Invent</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Conseil en transformation &amp; développement durable (entité de )</t>
+          <t>Conseil en Transformation &amp; Innovation Durable</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -3087,27 +3078,27 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Maëlle Bouvier</t>
+          <t>Cyril Garcia</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Director – Sustainable Future, Sustainability Director Invent France linkedin</t>
+          <t>Global Head of Sustainability Services &amp; Corporate Responsibility (ex-CEO Invent)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/fr-fr/services/developpement-durable/)</t>
+          <t>cyril.garcia@capgemini.com / contact.fr@capgemini.com</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/invent</t>
+          <t>https://www.linkedin.com/in/cyrilgarcia</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr-fr/services/developpement-durable/</t>
+          <t>https://www.capgemini.com/fr-fr/invent/</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3122,22 +3113,22 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme « Invent for Society » : proje</t>
+          <t>Programme « Invent for Society » &amp; Inclusion Numérique</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Positionner Ambition Campus comme vivier pour leurs équipes Sustainability/Net Zero et comme partenaire de programmes d’inclusion numérique et d’accès aux études d’ingénieurs/IT</t>
+          <t>Positionner Ambition Campus comme vivier pour leurs équipes Sustainability et partenaire d'accès aux filières IT/ingénieurs.</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr-fr/services/developpement-durable/ (offr</t>
+          <t>Solliciter un échange avec Cyril Garcia au siège 147 quai du Président Roosevelt (Issy-les-Moulineaux).</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3145,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Conseil en stratégie, bureau de Paris (14–16 rue des Capucines)</t>
+          <t>Conseil en Stratégie</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -3164,27 +3155,27 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Anne Corteggiano</t>
+          <t>Laurent Benarousse / Anne Corteggiano</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Director, Press Contact, Paris Office rolandberger</t>
+          <t>Managing Partner France / Director of External Affairs and Engagement</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www.rolandberger.com/fr/Locations/France/)</t>
+          <t>laurent.benarousse@rolandberger.com / anne.corteggiano@rolandberger.com</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/roland-berger-france</t>
+          <t>https://www.linkedin.com/in/laurentbenarousse</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>https://www.rolandberger.com/fr/Locations/France/</t>
+          <t>https://www.rolandberger.com/fr/</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3199,22 +3190,22 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Cabinet européen de référence, fortement</t>
+          <t>Partenariat « Club Dirigeants &amp; Égalité des Chances »</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Proposer un partenariat « club dirigeants &amp; égalité des chances » : tables rondes Roland Berger x Ambition Campus et parrainage de promotions de lycéens vers les filières économie/management rolandberger</t>
+          <t>Tables rondes Roland Berger x Ambition Campus et parrainage de promotions de lycéens vers les filières économie/management.</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www.rolandberger.com/fr/Locations/France/ (portail F</t>
+          <t>Contacter Laurent Benarousse et Anne Corteggiano au 14-16 rue des Capucines (Paris 2e).</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3222,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Cabinet d’avocats d’affaires français, très engagé en pro bono</t>
+          <t>Cabinet d'Avocats d'Affaires</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -3241,27 +3232,27 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Responsable Pro Bono / RSE (à préciser via contact Droits d’Urgence)</t>
+          <t>Myriam Epelbaum / Florence Haas</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Coordinateur·rice Pro Bono, partenariats avec Droits d’Urgence et Epic Foundation</t>
+          <t>Associée, Référente Gouvernance &amp; RSE / Associée, Comité de Direction &amp; Pro Bono</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..org/pro-bono/)</t>
+          <t>myriamepelbaum@bredinprat.com / florencehaas@bredinprat.com</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/bredin-prat</t>
+          <t>https://www.linkedin.com/in/myriam-epelbaum-71408824</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>https://www..org/pro-bono/</t>
+          <t>https://www.bredinprat.fr/engagements/</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3276,22 +3267,22 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Pro Bono structuré : permanences juridiq</t>
+          <t>Mécénat Pro Bono Structuré &amp; Mentorat Juridique</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Talents juridiques engagés » : pipeline de lycéens vers Droit Sorbonne/Assas, avec concours d’éloquence et mentorat assuré par les avocats Bredin Prat</t>
+          <t>Pitch « Talents juridiques engagés » : pipeline de lycéens vers Droit Sorbonne/Assas, concours d'éloquence et mentorat par les avocats.</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..org/pro-bono/ (partenariat Pro Bono Bredin Prat</t>
+          <t>Contacter Myriam Epelbaum et Florence Haas au 53 quai d'Orsay (Paris 7e).</t>
         </is>
       </c>
     </row>
@@ -3303,12 +3294,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Villey Maillot Brochier</t>
+          <t>Darrois Villey Maillot Brochier</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Cabinet d’avocats d’affaires de référence, indépendant à Paris</t>
+          <t>Cabinet d'Avocats d'Affaires</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
@@ -3318,27 +3309,27 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Responsable RSE / Charte RSE</t>
+          <t>Matthieu Brochier / Jean-Michel Darrois</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Responsable mise en œuvre de la charte RSE du cabinet</t>
+          <t>Associé Gérant, Référent Pro Bono &amp; Clinique du droit / Associé Fondateur</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/rse/)</t>
+          <t>mbrochier@darroisvilley.com / contact@darroisvilley.com</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/villey-maillot-brochier</t>
+          <t>https://www.linkedin.com/in/matthieu-brochier-39352010</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/rse/</t>
+          <t>https://www.darroisvilley.com/rse/</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3353,22 +3344,22 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Charte RSE structurée autour de la satis</t>
+          <t>Programme « Égalité des Chances &amp; Droit des Affaires »</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Co-construire un programme « égalité des chances &amp; Droit des affaires » : ateliers de découverte des carrières, coaching pour concours et immersion en cabinet pour lycéens Ambition Campus</t>
+          <t>Ateliers de découverte des carrières juridiques, coaching concours et immersion en cabinet pour lycéens d'excellence.</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/rse/ (charte RSE officielle)</t>
+          <t>Contacter Matthieu Brochier au 69 avenue Victor Hugo (Paris 16e).</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3376,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Cabinet d’avocats international, très fort engagement Pro Bono et égalité des chances</t>
+          <t>Cabinet d'Avocats International</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -3400,22 +3391,22 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Associé, co‑head de la pratique Pro Bono du bureau de Paris whitecase</t>
+          <t>Partner, Head of Paris Pro Bono Practice</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..fr/portfolio/white--case)</t>
+          <t>mpolkinghorne@whitecase.com / probono@whitecase.com</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/white-&amp;-case-paris</t>
+          <t>https://www.linkedin.com/in/michael-polkinghorne-30811b15</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>https://www..fr/portfolio/white--case</t>
+          <t>https://www.whitecase.com/locations/emea/france</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3430,22 +3421,22 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Pro Bono massif (4 500 h en 2020 sur ~65</t>
+          <t>Partenariat « Global Citizenship &amp; Éloquence »</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Global Citizenship &amp; concours d’éloquence » : mécénat financier + de compétences pour concours d’éloquence Ambition Campus, préparation aux carrières internationales (M&amp;A, arbitration) pour lycéens whitecase</t>
+          <t>Mécénat financier + de compétences pour concours d'éloquence Ambition Campus et préparation aux carrières internationales.</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..fr/portfolio/white--case (présentation engageme</t>
+          <t>Prendre contact avec Michael Polkinghorne au 19 place Vendôme (Paris 1er).</t>
         </is>
       </c>
     </row>
@@ -3455,40 +3446,44 @@
           <t>ENT-38</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Eurazeo</t>
+        </is>
+      </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Groupe d’investissement &amp; gestion d’actifs, forte plateforme ESG</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+          <t>Investissement &amp; Private Equity</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Finance, Private Equity &amp; Assurance</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Équipe ESG (contact esg@.com)</t>
+          <t>Sophie Flak</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Direction ESG / RSE, responsable reporting RSE et climat</t>
+          <t>Membre du Directoire, Managing Partner RSE, Sustainability &amp; Impact</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>esg@.com</t>
+          <t>sflak@eurazeo.com / esg@eurazeo.com</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/</t>
+          <t>https://www.linkedin.com/in/sophie-flak-3914a1</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/responsabilite/publications-esg</t>
+          <t>https://www.eurazeo.com/fr/responsabilite/publications-esg</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3503,22 +3498,22 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Stratégie ESG avancée : rapport O+ 2024,</t>
+          <t>Fonds de Bourses « Eurazeo - Ambition Campus »</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Proposer un fonds de bourses « – Ambition Campus » finançant prépas/Sciences Po, aligné sur leur priorité inclusion sociale et investissement durable, et pipeline de talents pour leurs équipes d’investissement</t>
+          <t>Bourses finançant prépas et Sciences Po, aligné sur leur stratégie ESG « O+ » et priorité inclusion sociale.</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/responsabilite/publications-esg (portail</t>
+          <t>Contacter Sophie Flak au siège 1 rue Georges Berger (Paris 17e).</t>
         </is>
       </c>
     </row>
@@ -3535,7 +3530,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Gestion d’actifs &amp; private equity, plateforme impact climat/biodiversité</t>
+          <t>Gestion d'Actifs &amp; Private Equity</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -3545,27 +3540,27 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Laure Villepelet</t>
+          <t>Mario Mitri / Pierre Abadie</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Head of ESG &amp; CSR Groupe docs.cfnews</t>
+          <t>Chief Sustainability Officer / Group Climate Director</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>lvillepelet@.com docs.cfnews</t>
+          <t>mmitri@tikehaucapital.com / pabadie@tikehaucapital.com</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/tikehau-capital</t>
+          <t>https://www.linkedin.com/in/mario-mitri</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/en/our-group/sustainability/publications</t>
+          <t>https://www.tikehaucapital.com/en/our-group/sustainability</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3580,22 +3575,22 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Approche « Sustainability by Design », p</t>
+          <t>Programme « Sustainability by Design &amp; Social Inclusion »</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Climate Action &amp; social inclusion » : financer bourses pour filières finance/climat, et co‑créer un track de recrutement de jeunes issus de QPV pour leurs équipes climate, biodiversité, private equity décarbonation docs.cfnews</t>
+          <t>Financer des bourses pour filières finance/climat et co-créer un track de recrutement de jeunes de QPV vers leurs équipes investissement.</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/en/our-group/sustainability/publications (p</t>
+          <t>Contacter Mario Mitri et Pierre Abadie au 32 rue de Monceau (Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -3605,40 +3600,44 @@
           <t>ENT-40</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr"/>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Ardian</t>
+        </is>
+      </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Private equity &amp; infrastructure, programme Sustainability structuré depuis 2008</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+          <t>Private Equity &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Finance, Private Equity &amp; Assurance</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Équipe Sustainability</t>
+          <t>Candice Brenet / Mathias Burghardt</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Sustainability Team (8 FTE), comité Sustainability</t>
+          <t>Managing Director, Head of Sustainability / Président de la Fondation Ardian</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/fr/sustainability)</t>
+          <t>candice.brenet@ardian.com / fondation@ardian.com</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/</t>
+          <t>https://www.linkedin.com/in/candice-brenet-4a2753</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/sustainability</t>
+          <t>https://www.ardian.com/fr/sustainability</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3653,22 +3652,22 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Intégration ESG dans 100% des fonds, qua</t>
+          <t>Mécénat Fondation Ardian &amp; Bourses de Mobilité Sociale</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Pitch « PE &amp; diversité des talents » : bourses et coaching vers Dauphine/ESSEC/HEC, pipeline de profils pour leurs équipes d’investissement et de portefeuille, aligné avec leur priorité égalité des chances</t>
+          <t>Bourses et coaching vers Dauphine, ESSEC, HEC, pipeline de profils pour leurs équipes d'investissement.</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/sustainability (vision Sustainability, p</t>
+          <t>Contacter Candice Brenet et l'équipe Fondation au 20 place Vendôme (Paris 1er).</t>
         </is>
       </c>
     </row>
@@ -3678,40 +3677,44 @@
           <t>ENT-41</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Amundi</t>
+        </is>
+      </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Gestion d’actifs, acteur de référence ESG en Europe</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Tier 3 - Grand Groupe &amp; Entreprise à Mission</t>
+          <t>Gestion d'Actifs (1er Asset Manager Européen)</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Tier 2 - Finance, Private Equity &amp; Assurance</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Direction ESG</t>
+          <t>Elodie Laugel / Caroline Le Meaux</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Responsable plan « Ambitions ESG 2025 »</t>
+          <t>Chief Responsible Investment Officer (Comex) / Global Head of ESG Research &amp; Engagement</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://legroupe..com/documentation-esg)</t>
+          <t>elodie.laugel@amundi.com / caroline.lemeaux@amundi.com</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/</t>
+          <t>https://www.linkedin.com/in/elodielaugel</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>https://legroupe..com/documentation-esg</t>
+          <t>https://legroupe.amundi.com/documentation-esg</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3726,22 +3729,22 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Convention Mécénat / Partenariat 847 Mds € d’actifs ESG (2021), approche </t>
+          <t>Programme « Finance Durable &amp; Égalité des Chances »</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Finance durable &amp; égalité des chances » : créer un programme de bourses climat/ESG pour lycéens destinant à la finance, et pipeline de stagiaires pour leurs équipes ESG/ETF/climat</t>
+          <t>Créer un programme de bourses climat/ESG pour lycéens se destinant à la finance et pipeline de stagiaires.</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://legroupe..com/documentation-esg (documentation ESG c</t>
+          <t>Contacter Elodie Laugel au siège 91-93 boulevard Pasteur (Paris 15e).</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3761,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Banque privée &amp; asset management, groupe financier européen indépendant</t>
+          <t>Banque Privée &amp; Asset Management</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -3768,27 +3771,27 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Direction RSE Groupe</t>
+          <t>Valentin Pernet</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Responsable démarche RSE (trois piliers)</t>
+          <t>Global Head of Sustainable Investment Solutions &amp; Fonds « Agir pour demain »</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/fr/engagements/)</t>
+          <t>valentin.pernet@oddo-bhf.com / contact@oddo-bhf.com</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/oddo-bhf</t>
+          <t>https://www.linkedin.com/in/valentin-pernet-87779b1b</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/engagements/</t>
+          <t>https://www.oddo-bhf.com/fr/engagements/</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3803,22 +3806,22 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Démarche RSE articulée autour de trois p</t>
+          <t>Mécénat via Fonds de Dotation « ODDO BHF Agir pour demain »</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Banque privée &amp; bourses d’excellence » : mécénat via fonds de dotation « Agir pour demain » ciblé sur lycéens Ambition Campus, avec parrainage vers les métiers de la banque privée et de la gestion d’actifs</t>
+          <t>Bourses d'excellence ciblées sur lycéens Ambition Campus et parrainage vers les métiers de la banque privée.</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/engagements/ (page engagements RSE group</t>
+          <t>Contacter Valentin Pernet au 12 boulevard de la Madeleine (Paris 9e).</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3838,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Gestion d’actifs, entité française de BlackRock, intégration systématique ESG</t>
+          <t>Gestion d'Actifs &amp; Marchés de Capitaux</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -3845,27 +3848,27 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Corporate Sustainability Controllers</t>
+          <t>Estelle Castres / Henri Chabadel</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Équipe Corporate Sustainability Controllers</t>
+          <t>Country Head France, Belux, Monaco / Chief Investment Officer France</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>corporate_sustainability_controllers@blackrock.com</t>
+          <t>estelle.castres@blackrock.com / henri.chabadel@blackrock.com</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/blackrock-france-sas</t>
+          <t>https://www.linkedin.com/in/estelle-castres-betzler-5881023</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>https://.fr/wp-content/uploads/2023/09/blackrock-france-sas-article-29-disclosure-2023.pdf</t>
+          <t>https://www.blackrock.com/fr</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3880,22 +3883,22 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Intégration des risques/opportunités ESG</t>
+          <t>Programme Bourses « BlackRock France - Ambition Campus »</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Global asset manager &amp; diversité » : créer un programme de bourses « BlackRock France – Ambition Campus » vers les filières finance internationale et marchés de capitaux, et pipeline de stagiaires pour leurs desks ESG/ETF</t>
+          <t>Bourses vers les filières finance internationale et marchés de capitaux, mentorat par les équipes d'investissement.</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://.fr/wp-content/uploads/2023/09/blackrock-france-sas-</t>
+          <t>Contacter Estelle Castres et Henri Chabadel au bureau de Paris (21 rue de la Ville-l'Évêque, Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -3907,12 +3910,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Allianz France</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Assurance, acteur majeur avec plan de transition net zero et labellisation RSE des agents</t>
+          <t>Assurance &amp; Gestion de Risques</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -3922,27 +3925,27 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Marie-Doha Besancenot</t>
+          <t>Marie-Doha Besancenot / Direction RSE</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Directrice RSE, Marque et Communication France rse-magazine</t>
+          <t>Directrice Marque, Communication &amp; RSE France</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..fr/qui-est-/-s-engage/notre-raison-d-etre/demarche-rse.html)</t>
+          <t>rse@allianz.fr / communication@allianz.fr</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/france</t>
+          <t>https://www.linkedin.com/company/allianz</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>https://www..fr/qui-est-/-s-engage/notre-raison-d-etre/demarche-rse.html</t>
+          <t>https://www.allianz.fr/qui-est-allianz/allianz-s-engage/notre-raison-d-etre/demarche-rse.html</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3957,22 +3960,22 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Démarche RSE articulée autour de économi</t>
+          <t>Mécénat Territorial &amp; Réseau d'Agents Engagés</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Assurance &amp; territoire » : mécénat territorial pour parrainer des lycées en zones de rénovation urbaine, engagements des agents labellisés RSE comme mentors pour les lycéens Ambition Campus</t>
+          <t>Mécénat territorial pour parrainer des lycées en zones de rénovation urbaine, engagement des collaborateurs comme mentors.</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..fr/qui-est-/-s-engage/notre-raison-d-etre/demar</t>
+          <t>Cibler la Direction RSE et Communication à la Tour Allianz One (Paris La Défense).</t>
         </is>
       </c>
     </row>
@@ -3982,10 +3985,14 @@
           <t>ENT-45</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Groupama</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Mutuelle d’assurance, stratégie RSE structurante avec label AFNOR « Engagé RSE »</t>
+          <t>Mutuelle d'Assurance &amp; Banque</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -3995,27 +4002,27 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Équipe Durabilité Groupe</t>
+          <t>François Coste / Direction Durabilité</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Direction Durabilité / RSE Groupe</t>
+          <t>Directeur Groupe Durabilité / Sustainability Groupama</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/fr/engagements-rse/)</t>
+          <t>francois.coste@groupama.com / rse@groupama.com</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/</t>
+          <t>https://www.linkedin.com/in/francois-coste-groupama</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/engagements-rse/</t>
+          <t>https://www.groupama.com/fr/engagements-rse/</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -4030,22 +4037,22 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme de labellisation AFNOR « Engag</t>
+          <t>Mécénat Territorial &amp; Inclusion des Jeunes</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Assureur de proximité &amp; égalité des chances » : mécénat territorial pour soutenir les lycées partenaires Ambition Campus en zones rurales/périurbaines, avec interventions de collaborateurs sur les métiers de l’assurance et de la gestion des risques</t>
+          <t>Soutien aux lycées partenaires Ambition Campus en zones périurbaines et rurales, interventions sur la gestion des risques.</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/engagements-rse/ (engagements RSE groupe</t>
+          <t>Contacter François Coste au siège 8-10 rue d'Astorg (Paris 8e).</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4069,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Groupe agroalimentaire, Société à Mission &amp; B Corp mondiale</t>
+          <t>Agroalimentaire (Société à Mission &amp; B Corp)</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -4072,27 +4079,27 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Direction Impact Journey / Mission</t>
+          <t>Nathalie Alquier / Thomas Kyriaco</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Responsable Danone Impact Journey et comité de mission danone</t>
+          <t>Chief Sustainability Officer / Directeur RSE &amp; Impact Journey</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/fr/engagements.html)</t>
+          <t>nathalie.alquier@danone.com / thomas.kyriaco@danone.com</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/danone</t>
+          <t>https://www.linkedin.com/in/nathalie-alquier-591b721</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/engagements.html</t>
+          <t>https://www.danone.com/fr/engagements.html</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -4107,22 +4114,22 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Statut Société à Mission (première entre</t>
+          <t>Partenariat « Santé, Alimentation &amp; Mobilité Sociale »</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Santé par l’alimentation &amp; mobilité sociale » : bourses pour filières médecine, nutrition, économie/gestion, et programme de mentorat pour lycéens Ambition Campus vers les métiers du droit/finance/industrie agroalimentaire chez Danone</t>
+          <t>Bourses pour filières médecine, nutrition, économie/gestion et mentorat vers les métiers juridiques/financiers de Danone.</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/engagements.html (feuille de route Danon</t>
+          <t>Contacter Nathalie Alquier et Thomas Kyriaco au 17 boulevard Haussmann (Paris 9e).</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4146,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Technologies de l’énergie &amp; automatisation, leader mondial du développement durable</t>
+          <t>Technologies de l'Énergie &amp; Automatisation</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -4149,27 +4156,27 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Direction Développement Durable France</t>
+          <t>Gilles Vermot Desroches</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Responsable programme Schneider Sustainability Impact (SSI)</t>
+          <t>Chief Sustainability Officer &amp; Délégué Général Fondation Schneider Electric</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/fr/fr/about-us/sustainability/)</t>
+          <t>gilles.vermot-desroches@se.com</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/schneider-electric</t>
+          <t>https://www.linkedin.com/in/gilles-vermot-desroches-0363212</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr/fr/about-us/sustainability/</t>
+          <t>https://www.se.com/fr/fr/about-us/sustainability/</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
@@ -4184,22 +4191,22 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Programme Schneider Sustainability Impac</t>
+          <t>Programme « Énergie Verte, Tech &amp; Inclusion »</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Énergie verte &amp; inclusion » : partenariat mêlant visites de sites, hackathons énergie pour lycéens Ambition Campus et pipeline de talents pour les métiers d’ingénieur et de data dans la transition énergétique</t>
+          <t>Partenariat mêlant visites de sites, hackathons énergie pour lycéens et pipeline de talents pour métiers d'ingénieur.</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr/fr/about-us/sustainability/ (portail glo</t>
+          <t>Contacter Gilles Vermot Desroches au siège 35 rue Joseph Monier (Rueil-Malmaison).</t>
         </is>
       </c>
     </row>
@@ -4211,12 +4218,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>(Groupe)</t>
+          <t>Capgemini (Groupe)</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Services numériques &amp; ingénierie, forte stratégie climat et Net Zero</t>
+          <t>Services Numériques &amp; Ingénierie</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -4226,27 +4233,27 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Direction Développement Durable Groupe</t>
+          <t>Cyril Garcia</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Responsable stratégie climat et Net Zero (par ex. VP Conseil Développement Durable &amp; Transition énergétique)</t>
+          <t>Global Head of Sustainability Services &amp; Corporate Responsibility (Comex)</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>via direction RSE (https://www..com/fr-fr/services/developpement-durable/)</t>
+          <t>cyril.garcia@capgemini.com / contact.fr@capgemini.com</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/(groupe)</t>
+          <t>https://www.linkedin.com/in/cyrilgarcia</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>https://www..com/fr-fr/services/developpement-durable/</t>
+          <t>https://www.capgemini.com/fr-fr/services/developpement-durable/</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -4261,22 +4268,22 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>Convention Mécénat / Partenariat Engagements Net Zero, objectifs de réduc</t>
+          <t>Programme « Tech, Numérique Inclusif &amp; Égalité des Chances »</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Pitch « Tech &amp; égalité des chances » : mécénat pour équiper lycéens en matériel numérique, bootcamps IA/développement avec consultants , et pipeline de profils pour les filières ingénieurs/IT du groupe</t>
+          <t>Mécénat pour équiper lycéens en matériel numérique, bootcamps IA/code et pipeline pour filières ingénieurs/IT.</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>À qualifier &amp; contacter</t>
+          <t>À contacter</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>Proposer une convention de mécénat 2026-2027 et masterclass métier. Source RSE : https://www..com/fr-fr/services/developpement-durable/ (déve</t>
+          <t>Contacter Cyril Garcia au siège 11 rue de Tilsitt (Paris 17e) ou campus Issy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prospection : vérification OSINT des contacts (Firecrawl + Perplexity) et correction des LinkedIn
- scripts/verify_contacts_osint.py : pipeline en 4 phases (firecrawl / perplexity / report / apply),
  recherche Google site:linkedin.com/in par contact, confirmation nominative des postes par Perplexity,
  contrôle du format d'email par domaine ; cache brut gitignoré, retry sur 429 et erreurs réseau
- 77 contacts analysés : 6 URLs LinkedIn correctes, 69 corrigées (slug inventé), 2 introuvables ;
  64 corrections appliquées automatiquement (prénom + nom + entreprise concordants)
- update_initial_data.py : un LinkedIn par contact (plus de partage de l'URL du 1er contact)
- Base CSV/XLSX et initialData.json régénérés ; rapport et CSV de vérification datés du 2026-09-03
- Emails non vérifiés en SMTP (format seulement) : nécessite Hunter / Dropcontact / Reoon

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prospection/entreprises/entreprises_database.xlsx
+++ b/prospection/entreprises/entreprises_database.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Master_Entreprises" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master_Entreprises" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -86,13 +89,19 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -114,19 +123,19 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -629,7 +638,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/adelaide-de-tourtier</t>
+          <t>https://www.linkedin.com/in/adelaide-de-tourtier-audras-4a423a1 / https://www.linkedin.com/in/candice-galopeau-16a6b291</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -706,7 +715,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/guilene-bertin-perri</t>
+          <t>https://www.linkedin.com/in/guil%C3%A8ne-bertin-60298b91 / https://www.linkedin.com/in/bertrand-boisselier-63b7176</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -783,7 +792,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bouchra-aliouat</t>
+          <t>https://www.linkedin.com/in/bouchra-aliouat-b62a0012 / https://www.linkedin.com/in/khalid-hima-66712b7b</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -860,7 +869,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/fabienne-marqueste</t>
+          <t>https://www.linkedin.com/in/fabienne-marqueste-32864526 / https://www.linkedin.com/in/oranetribouley</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -937,7 +946,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/marie-anne-brin</t>
+          <t>https://www.linkedin.com/in/marie-anne-brin-14330131</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1014,7 +1023,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/helene-cambournac</t>
+          <t>https://www.linkedin.com/in/helene-cambournac / https://www.linkedin.com/in/cedricbaecher</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1091,7 +1100,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/patrick-dupoux-51543b</t>
+          <t>https://www.linkedin.com/in/patrick-dupoux-51543b / https://www.linkedin.com/in/thomas-payen-2581472b</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1168,7 +1177,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/alain-imbert-4720235</t>
+          <t>https://www.linkedin.com/in/alain-imbert-4720235 / https://www.linkedin.com/in/christopherohel</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1322,7 +1331,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/anne-pointet</t>
+          <t>https://www.linkedin.com/in/anne-pointet / https://www.linkedin.com/in/isabelle-giordano</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1399,7 +1408,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/tanguy-claquin</t>
+          <t>https://www.linkedin.com/in/tanguy-claquin-30ba124a</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1476,7 +1485,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/groupe-bpce</t>
+          <t>https://www.linkedin.com/company/groupe-bpce / https://www.linkedin.com/in/virginienormand</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1553,7 +1562,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/sophie-de-nadaillac-98305711</t>
+          <t>https://www.linkedin.com/in/sophie-de-nadaillac</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1707,7 +1716,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/carole-malinvaud-091a1b18</t>
+          <t>https://www.linkedin.com/in/carole-malinvaud-73472335</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1784,7 +1793,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/fabienne-haas-36b12a32</t>
+          <t>https://www.linkedin.com/in/fabienne-haas-bb1b15a / https://www.linkedin.com/in/emmanuelle-barbara-3a178860</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1861,7 +1870,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/charles-henri-boeringer-031a002</t>
+          <t>https://www.linkedin.com/in/charles-henri-boeringer-42566342 / https://www.linkedin.com/in/mathieu-remy-398a375</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -2092,7 +2101,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/enericlopez</t>
+          <t>https://www.linkedin.com/in/elopezfr</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -2246,7 +2255,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/arnaud-bosom</t>
+          <t>https://www.linkedin.com/in/arnaud-bosom / https://www.linkedin.com/in/sophie-danis-verloove</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2323,7 +2332,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/anne-laure-thomas-5b72224</t>
+          <t>https://www.linkedin.com/in/anne-laure-thomas-b056581</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2400,7 +2409,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/alexandre-boquel-128a3818</t>
+          <t>https://www.linkedin.com/in/alexandre-boquel-33277910a / https://www.linkedin.com/in/antoine-arnault-lvmh</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2477,7 +2486,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/patrizia-gatti-gregori-43615410</t>
+          <t>https://www.linkedin.com/in/patrizia-gatti-a659276a</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2554,7 +2563,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/claire-pedini-1b641a23</t>
+          <t>https://www.linkedin.com/in/claire-pedini-652b0610b</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2631,7 +2640,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/anatole-de-la-brosse-b02441</t>
+          <t>https://www.linkedin.com/in/anatole-de-la-brosse-2110666</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2708,7 +2717,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/axelle-paquer-7b1990</t>
+          <t>https://www.linkedin.com/in/axellepaquer / https://www.linkedin.com/in/s%25C3%25A9bastien-gu%25C3%25A9chot</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2785,7 +2794,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/vincent-bamberger-155097</t>
+          <t>https://www.linkedin.com/in/vincent-bamberger-5a4723133 / https://www.linkedin.com/in/florentnanse</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2862,7 +2871,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bruno-despujol-5593892</t>
+          <t>https://www.linkedin.com/in/bruno-despujol-8224197</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2939,7 +2948,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/delphine-bourrilly-8208945</t>
+          <t>https://www.linkedin.com/in/delphine-bourrilly-8208945 / https://www.linkedin.com/in/nicolaslioliakis</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -3016,7 +3025,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/david-vidal-5764b8</t>
+          <t>https://www.linkedin.com/in/david-vidal-0ab7427 / https://www.linkedin.com/in/kai-bandilla-35b3b19 / https://www.linkedin.com/in/camille-fouillade-26711267</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -3093,7 +3102,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/cyrilgarcia</t>
+          <t>https://www.linkedin.com/in/cyrilgarcia1</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -3170,7 +3179,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/laurentbenarousse</t>
+          <t>https://www.linkedin.com/in/laurent-benarousse / https://www.linkedin.com/in/anne-corteggiano-1a06ba46</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -3247,7 +3256,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/myriam-epelbaum-71408824</t>
+          <t>https://www.linkedin.com/in/myriam-epelbaum-a2088576 / https://www.linkedin.com/in/florence-haas-368b936b</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -3324,7 +3333,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/matthieu-brochier-39352010</t>
+          <t>https://www.linkedin.com/in/matthieu-brochier-baaa3887</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -3401,7 +3410,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/michael-polkinghorne-30811b15</t>
+          <t>https://www.linkedin.com/in/michaelpolkinghorne</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -3555,7 +3564,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mario-mitri</t>
+          <t>https://www.linkedin.com/in/mario-mitri / https://www.linkedin.com/in/pierreabadie</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -3632,7 +3641,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/candice-brenet-4a2753</t>
+          <t>https://www.linkedin.com/in/candice-brenet / https://www.linkedin.com/in/mathias-burghardt</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -3709,7 +3718,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/elodielaugel</t>
+          <t>https://www.linkedin.com/in/elodielaugel / https://www.linkedin.com/in/carolinelemeauxlambert</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -3786,7 +3795,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/valentin-pernet-87779b1b</t>
+          <t>https://www.linkedin.com/in/valentin-pernet-6396744b</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -3863,7 +3872,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/estelle-castres-betzler-5881023</t>
+          <t>https://www.linkedin.com/in/estelle-castres-49ab9419 / https://www.linkedin.com/in/henri-chabadel-374419110</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -3940,7 +3949,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/allianz</t>
+          <t>https://www.linkedin.com/in/mdohabesancenot</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -4094,7 +4103,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/nathalie-alquier-591b721</t>
+          <t>https://www.linkedin.com/in/nathalie-alquier-9063499a / https://www.linkedin.com/in/thomas-kyriaco-4211a05</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -4171,7 +4180,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/gilles-vermot-desroches-0363212</t>
+          <t>https://www.linkedin.com/in/gilles-vermot-desroches</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -4248,7 +4257,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/cyrilgarcia</t>
+          <t>https://www.linkedin.com/in/cyrilgarcia1</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">

</xml_diff>